<commit_message>
:sparkles: a good report of predictive analysis
</commit_message>
<xml_diff>
--- a/TCC II/dados/dicionario de dados campos obrigatorios.xlsx
+++ b/TCC II/dados/dicionario de dados campos obrigatorios.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\iasmi\OneDrive\Documents\UFES\2025-1\TCC II\dados\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\iasmi\OneDrive\Documents\UFES\2025-1\TCC II\srag_tcc\TCC II\dados\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5C786809-6B49-4A9F-8C08-71FAABA4250A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BA3B612B-6FB2-43E5-B481-A2AC27F41B70}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{E08B2D45-4FCA-4544-BDE7-A7BAB001B13E}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="143" uniqueCount="133">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="172" uniqueCount="156">
   <si>
     <t>Nome do campo</t>
   </si>
@@ -610,6 +610,81 @@
 UF do usuário. 
 * Federal - abre tabela com todas as UF que possuam unidades 
 cadastradas no sistema. </t>
+  </si>
+  <si>
+    <t xml:space="preserve">12-Data de nascimento </t>
+  </si>
+  <si>
+    <t>Data de nascimento 
+do paciente.</t>
+  </si>
+  <si>
+    <t>Data deve ser &lt;= a data dos primeiros sintomas.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DT_NASC </t>
+  </si>
+  <si>
+    <t>35-Fatores de risco</t>
+  </si>
+  <si>
+    <t>Paciente apresenta 
+algum fator de risco</t>
+  </si>
+  <si>
+    <t>FATOR_RISC</t>
+  </si>
+  <si>
+    <t>77- Data do Resultado</t>
+  </si>
+  <si>
+    <t>Data do Resultado do Teste Sorológico</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Data deve ser maior ou igual a 75- Data da Coleta </t>
+  </si>
+  <si>
+    <t>DT_RES</t>
+  </si>
+  <si>
+    <t xml:space="preserve">EVOLUCAO </t>
+  </si>
+  <si>
+    <t xml:space="preserve">DT_EVOLUCA </t>
+  </si>
+  <si>
+    <t>Data da alta ou do óbito deve ser &gt; ou = a data dos primeiros sintomas e &lt;= a data da digitação (atual). Habilitado se campo 80- Evolução do caso = 1 ou 2.</t>
+  </si>
+  <si>
+    <t>Data da alta ou 
+óbito</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Evolução do caso </t>
+  </si>
+  <si>
+    <t>1-Cura 
+2-Óbito 
+3- Óbito por outras causas 
+9-Ignorado</t>
+  </si>
+  <si>
+    <t xml:space="preserve">80–Evolução do caso </t>
+  </si>
+  <si>
+    <t xml:space="preserve">81–Data da alta ou óbito </t>
+  </si>
+  <si>
+    <t xml:space="preserve">83- Número D.O </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Número da Declaração de Óbito </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Habilitado se o campo 80- Evolução do caso = 2 ou 3 </t>
+  </si>
+  <si>
+    <t xml:space="preserve">NU_DO </t>
   </si>
 </sst>
 </file>
@@ -633,12 +708,24 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="12">
@@ -778,19 +865,79 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="23">
+  <cellXfs count="28">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="9" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
@@ -800,51 +947,6 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1160,517 +1262,623 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C2713F42-569F-421A-AAD9-F9B7A7929CC4}">
-  <dimension ref="A1:F27"/>
+  <dimension ref="A1:F33"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="25.44140625" style="21" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="13.21875" style="22" customWidth="1"/>
-    <col min="3" max="3" width="19" style="22" customWidth="1"/>
-    <col min="4" max="4" width="41.44140625" style="22" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="64.33203125" style="21" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="15.33203125" style="22" customWidth="1"/>
+    <col min="1" max="1" width="25.44140625" style="5" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="13.21875" style="6" customWidth="1"/>
+    <col min="3" max="3" width="19" style="6" customWidth="1"/>
+    <col min="4" max="4" width="41.44140625" style="6" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="64.33203125" style="5" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="15.33203125" style="6" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="5" t="s">
+      <c r="A1" s="25" t="s">
         <v>129</v>
       </c>
-      <c r="B1" s="6"/>
-      <c r="C1" s="6"/>
-      <c r="D1" s="6"/>
-      <c r="E1" s="6"/>
-      <c r="F1" s="7"/>
+      <c r="B1" s="26"/>
+      <c r="C1" s="26"/>
+      <c r="D1" s="26"/>
+      <c r="E1" s="26"/>
+      <c r="F1" s="27"/>
     </row>
     <row r="2" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="8" t="s">
+      <c r="A2" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="9" t="s">
+      <c r="B2" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="C2" s="9" t="s">
+      <c r="C2" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="D2" s="9" t="s">
+      <c r="D2" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="E2" s="10" t="s">
+      <c r="E2" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="F2" s="11" t="s">
+      <c r="F2" s="4" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="3" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A3" s="12" t="s">
+      <c r="A3" s="16" t="s">
         <v>130</v>
       </c>
-      <c r="B3" s="13" t="s">
+      <c r="B3" s="17" t="s">
         <v>6</v>
       </c>
-      <c r="C3" s="14"/>
-      <c r="D3" s="13" t="s">
+      <c r="C3" s="18"/>
+      <c r="D3" s="17" t="s">
         <v>131</v>
       </c>
-      <c r="E3" s="13" t="s">
+      <c r="E3" s="17" t="s">
         <v>7</v>
       </c>
-      <c r="F3" s="15" t="s">
+      <c r="F3" s="19" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="4" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A4" s="3" t="s">
+      <c r="A4" s="20" t="s">
         <v>9</v>
       </c>
-      <c r="B4" s="1" t="s">
+      <c r="B4" s="21" t="s">
         <v>6</v>
       </c>
-      <c r="C4" s="2"/>
-      <c r="D4" s="1" t="s">
+      <c r="C4" s="22"/>
+      <c r="D4" s="21" t="s">
         <v>10</v>
       </c>
-      <c r="E4" s="1" t="s">
+      <c r="E4" s="21" t="s">
         <v>11</v>
       </c>
-      <c r="F4" s="4" t="s">
+      <c r="F4" s="23" t="s">
         <v>12</v>
       </c>
     </row>
     <row r="5" spans="1:6" ht="129.6" x14ac:dyDescent="0.3">
-      <c r="A5" s="3" t="s">
+      <c r="A5" s="20" t="s">
         <v>13</v>
       </c>
-      <c r="B5" s="2" t="s">
+      <c r="B5" s="22" t="s">
         <v>14</v>
       </c>
-      <c r="C5" s="1" t="s">
+      <c r="C5" s="21" t="s">
         <v>16</v>
       </c>
-      <c r="D5" s="1" t="s">
+      <c r="D5" s="21" t="s">
         <v>15</v>
       </c>
-      <c r="E5" s="1" t="s">
+      <c r="E5" s="21" t="s">
         <v>132</v>
       </c>
-      <c r="F5" s="4" t="s">
+      <c r="F5" s="23" t="s">
         <v>17</v>
       </c>
     </row>
     <row r="6" spans="1:6" ht="144" x14ac:dyDescent="0.3">
-      <c r="A6" s="3" t="s">
+      <c r="A6" s="20" t="s">
         <v>18</v>
       </c>
-      <c r="B6" s="2" t="s">
+      <c r="B6" s="22" t="s">
         <v>19</v>
       </c>
-      <c r="C6" s="1" t="s">
+      <c r="C6" s="21" t="s">
         <v>20</v>
       </c>
-      <c r="D6" s="1" t="s">
+      <c r="D6" s="21" t="s">
         <v>21</v>
       </c>
-      <c r="E6" s="1" t="s">
+      <c r="E6" s="21" t="s">
         <v>23</v>
       </c>
-      <c r="F6" s="4" t="s">
+      <c r="F6" s="23" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="7" spans="1:6" ht="115.2" x14ac:dyDescent="0.3">
-      <c r="A7" s="3" t="s">
+      <c r="A7" s="20" t="s">
         <v>24</v>
       </c>
-      <c r="B7" s="2" t="s">
+      <c r="B7" s="22" t="s">
         <v>25</v>
       </c>
-      <c r="C7" s="1" t="s">
+      <c r="C7" s="21" t="s">
         <v>26</v>
       </c>
-      <c r="D7" s="1" t="s">
+      <c r="D7" s="21" t="s">
         <v>27</v>
       </c>
-      <c r="E7" s="1" t="s">
+      <c r="E7" s="21" t="s">
         <v>28</v>
       </c>
-      <c r="F7" s="4" t="s">
+      <c r="F7" s="23" t="s">
         <v>29</v>
       </c>
     </row>
     <row r="8" spans="1:6" ht="72" x14ac:dyDescent="0.3">
-      <c r="A8" s="3" t="s">
+      <c r="A8" s="20" t="s">
         <v>30</v>
       </c>
-      <c r="B8" s="2" t="s">
+      <c r="B8" s="22" t="s">
         <v>31</v>
       </c>
-      <c r="C8" s="1" t="s">
+      <c r="C8" s="21" t="s">
         <v>32</v>
       </c>
-      <c r="D8" s="1" t="s">
+      <c r="D8" s="21" t="s">
         <v>33</v>
       </c>
-      <c r="E8" s="1" t="s">
+      <c r="E8" s="21" t="s">
         <v>34</v>
       </c>
-      <c r="F8" s="4" t="s">
+      <c r="F8" s="23" t="s">
         <v>35</v>
       </c>
     </row>
     <row r="9" spans="1:6" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="A9" s="3" t="s">
+      <c r="A9" s="20" t="s">
         <v>36</v>
       </c>
-      <c r="B9" s="2" t="s">
+      <c r="B9" s="22" t="s">
         <v>37</v>
       </c>
-      <c r="C9" s="1" t="s">
+      <c r="C9" s="21" t="s">
         <v>38</v>
       </c>
-      <c r="D9" s="1" t="s">
+      <c r="D9" s="21" t="s">
         <v>39</v>
       </c>
-      <c r="E9" s="1" t="s">
+      <c r="E9" s="21" t="s">
         <v>40</v>
       </c>
-      <c r="F9" s="4" t="s">
+      <c r="F9" s="23" t="s">
         <v>41</v>
       </c>
     </row>
     <row r="10" spans="1:6" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A10" s="3" t="s">
+      <c r="A10" s="20" t="s">
         <v>42</v>
       </c>
-      <c r="B10" s="2" t="s">
+      <c r="B10" s="22" t="s">
         <v>31</v>
       </c>
-      <c r="C10" s="1" t="s">
+      <c r="C10" s="21" t="s">
         <v>32</v>
       </c>
-      <c r="D10" s="1" t="s">
+      <c r="D10" s="21" t="s">
         <v>43</v>
       </c>
-      <c r="E10" s="1" t="s">
+      <c r="E10" s="21" t="s">
         <v>44</v>
       </c>
-      <c r="F10" s="4" t="s">
+      <c r="F10" s="23" t="s">
         <v>45</v>
       </c>
     </row>
     <row r="11" spans="1:6" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="A11" s="3" t="s">
+      <c r="A11" s="20" t="s">
         <v>46</v>
       </c>
-      <c r="B11" s="2" t="s">
+      <c r="B11" s="22" t="s">
         <v>37</v>
       </c>
-      <c r="C11" s="1" t="s">
+      <c r="C11" s="21" t="s">
         <v>47</v>
       </c>
-      <c r="D11" s="1" t="s">
+      <c r="D11" s="21" t="s">
         <v>48</v>
       </c>
-      <c r="E11" s="1"/>
-      <c r="F11" s="4" t="s">
+      <c r="E11" s="21"/>
+      <c r="F11" s="23" t="s">
         <v>49</v>
       </c>
     </row>
     <row r="12" spans="1:6" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A12" s="3" t="s">
+      <c r="A12" s="20" t="s">
         <v>50</v>
       </c>
-      <c r="B12" s="2" t="s">
+      <c r="B12" s="22" t="s">
         <v>51</v>
       </c>
-      <c r="C12" s="2"/>
-      <c r="D12" s="1" t="s">
+      <c r="C12" s="22"/>
+      <c r="D12" s="21" t="s">
         <v>52</v>
       </c>
-      <c r="E12" s="1"/>
-      <c r="F12" s="4" t="s">
+      <c r="E12" s="21"/>
+      <c r="F12" s="23" t="s">
         <v>53</v>
       </c>
     </row>
     <row r="13" spans="1:6" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A13" s="3" t="s">
+      <c r="A13" s="20" t="s">
         <v>54</v>
       </c>
-      <c r="B13" s="2" t="s">
+      <c r="B13" s="22" t="s">
         <v>55</v>
       </c>
-      <c r="C13" s="1" t="s">
+      <c r="C13" s="21" t="s">
         <v>66</v>
       </c>
-      <c r="D13" s="1" t="s">
+      <c r="D13" s="21" t="s">
         <v>56</v>
       </c>
-      <c r="E13" s="1"/>
-      <c r="F13" s="16" t="s">
+      <c r="E13" s="21"/>
+      <c r="F13" s="24" t="s">
         <v>57</v>
       </c>
     </row>
     <row r="14" spans="1:6" ht="129.6" x14ac:dyDescent="0.3">
-      <c r="A14" s="3" t="s">
+      <c r="A14" s="20" t="s">
         <v>58</v>
       </c>
-      <c r="B14" s="2" t="s">
+      <c r="B14" s="22" t="s">
         <v>59</v>
       </c>
-      <c r="C14" s="2"/>
-      <c r="D14" s="1" t="s">
+      <c r="C14" s="22"/>
+      <c r="D14" s="21" t="s">
         <v>60</v>
       </c>
-      <c r="E14" s="1" t="s">
+      <c r="E14" s="21" t="s">
         <v>61</v>
       </c>
-      <c r="F14" s="4" t="s">
+      <c r="F14" s="23" t="s">
         <v>62</v>
       </c>
     </row>
     <row r="15" spans="1:6" ht="216" x14ac:dyDescent="0.3">
-      <c r="A15" s="3" t="s">
+      <c r="A15" s="20" t="s">
         <v>63</v>
       </c>
-      <c r="B15" s="2" t="s">
+      <c r="B15" s="22" t="s">
         <v>64</v>
       </c>
-      <c r="C15" s="1" t="s">
+      <c r="C15" s="21" t="s">
         <v>65</v>
       </c>
-      <c r="D15" s="2"/>
-      <c r="E15" s="1" t="s">
+      <c r="D15" s="22"/>
+      <c r="E15" s="21" t="s">
         <v>67</v>
       </c>
-      <c r="F15" s="4" t="s">
+      <c r="F15" s="23" t="s">
         <v>68</v>
       </c>
     </row>
     <row r="16" spans="1:6" ht="115.2" x14ac:dyDescent="0.3">
-      <c r="A16" s="3" t="s">
+      <c r="A16" s="20" t="s">
         <v>69</v>
       </c>
-      <c r="B16" s="2" t="s">
+      <c r="B16" s="22" t="s">
         <v>64</v>
       </c>
-      <c r="C16" s="1" t="s">
+      <c r="C16" s="21" t="s">
         <v>70</v>
       </c>
-      <c r="D16" s="1" t="s">
+      <c r="D16" s="21" t="s">
         <v>71</v>
       </c>
-      <c r="E16" s="1" t="s">
+      <c r="E16" s="21" t="s">
         <v>72</v>
       </c>
-      <c r="F16" s="4" t="s">
+      <c r="F16" s="23" t="s">
         <v>73</v>
       </c>
     </row>
-    <row r="17" spans="1:6" ht="187.2" x14ac:dyDescent="0.3">
-      <c r="A17" s="3" t="s">
+    <row r="17" spans="1:6" ht="172.8" x14ac:dyDescent="0.3">
+      <c r="A17" s="20" t="s">
         <v>74</v>
       </c>
-      <c r="B17" s="2" t="s">
+      <c r="B17" s="22" t="s">
         <v>14</v>
       </c>
-      <c r="C17" s="1" t="s">
+      <c r="C17" s="21" t="s">
         <v>75</v>
       </c>
-      <c r="D17" s="1" t="s">
+      <c r="D17" s="21" t="s">
         <v>76</v>
       </c>
-      <c r="E17" s="1"/>
-      <c r="F17" s="4" t="s">
+      <c r="E17" s="21"/>
+      <c r="F17" s="23" t="s">
         <v>77</v>
       </c>
     </row>
     <row r="18" spans="1:6" ht="86.4" x14ac:dyDescent="0.3">
-      <c r="A18" s="3" t="s">
+      <c r="A18" s="20" t="s">
         <v>78</v>
       </c>
-      <c r="B18" s="2" t="s">
+      <c r="B18" s="22" t="s">
         <v>79</v>
       </c>
-      <c r="C18" s="1" t="s">
+      <c r="C18" s="21" t="s">
         <v>80</v>
       </c>
-      <c r="D18" s="1" t="s">
+      <c r="D18" s="21" t="s">
         <v>81</v>
       </c>
-      <c r="E18" s="1"/>
-      <c r="F18" s="4" t="s">
+      <c r="E18" s="21"/>
+      <c r="F18" s="23" t="s">
         <v>82</v>
       </c>
     </row>
     <row r="19" spans="1:6" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A19" s="3" t="s">
+      <c r="A19" s="20" t="s">
         <v>83</v>
       </c>
-      <c r="B19" s="2" t="s">
+      <c r="B19" s="22" t="s">
         <v>84</v>
       </c>
-      <c r="C19" s="1" t="s">
+      <c r="C19" s="21" t="s">
         <v>85</v>
       </c>
-      <c r="D19" s="1" t="s">
+      <c r="D19" s="21" t="s">
         <v>86</v>
       </c>
-      <c r="E19" s="1" t="s">
+      <c r="E19" s="21" t="s">
         <v>87</v>
       </c>
-      <c r="F19" s="4" t="s">
+      <c r="F19" s="23" t="s">
         <v>88</v>
       </c>
     </row>
     <row r="20" spans="1:6" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="A20" s="3" t="s">
+      <c r="A20" s="20" t="s">
         <v>89</v>
       </c>
-      <c r="B20" s="2" t="s">
+      <c r="B20" s="22" t="s">
         <v>14</v>
       </c>
-      <c r="C20" s="1" t="s">
+      <c r="C20" s="21" t="s">
         <v>16</v>
       </c>
-      <c r="D20" s="1" t="s">
+      <c r="D20" s="21" t="s">
         <v>90</v>
       </c>
-      <c r="E20" s="1" t="s">
+      <c r="E20" s="21" t="s">
         <v>91</v>
       </c>
-      <c r="F20" s="4" t="s">
+      <c r="F20" s="23" t="s">
         <v>92</v>
       </c>
     </row>
     <row r="21" spans="1:6" ht="158.4" x14ac:dyDescent="0.3">
-      <c r="A21" s="3" t="s">
+      <c r="A21" s="20" t="s">
         <v>93</v>
       </c>
-      <c r="B21" s="2" t="s">
+      <c r="B21" s="22" t="s">
         <v>94</v>
       </c>
-      <c r="C21" s="1" t="s">
+      <c r="C21" s="21" t="s">
         <v>96</v>
       </c>
-      <c r="D21" s="1" t="s">
+      <c r="D21" s="21" t="s">
         <v>95</v>
       </c>
-      <c r="E21" s="1" t="s">
+      <c r="E21" s="21" t="s">
         <v>97</v>
       </c>
-      <c r="F21" s="4" t="s">
+      <c r="F21" s="23" t="s">
         <v>98</v>
       </c>
     </row>
     <row r="22" spans="1:6" ht="72" x14ac:dyDescent="0.3">
-      <c r="A22" s="3" t="s">
+      <c r="A22" s="20" t="s">
         <v>99</v>
       </c>
-      <c r="B22" s="2" t="s">
+      <c r="B22" s="22" t="s">
         <v>100</v>
       </c>
-      <c r="C22" s="1" t="s">
+      <c r="C22" s="21" t="s">
         <v>101</v>
       </c>
-      <c r="D22" s="1" t="s">
+      <c r="D22" s="21" t="s">
         <v>102</v>
       </c>
-      <c r="E22" s="1" t="s">
+      <c r="E22" s="21" t="s">
         <v>103</v>
       </c>
-      <c r="F22" s="4" t="s">
+      <c r="F22" s="23" t="s">
         <v>104</v>
       </c>
     </row>
     <row r="23" spans="1:6" ht="86.4" x14ac:dyDescent="0.3">
-      <c r="A23" s="3" t="s">
+      <c r="A23" s="20" t="s">
         <v>105</v>
       </c>
-      <c r="B23" s="2" t="s">
+      <c r="B23" s="22" t="s">
         <v>106</v>
       </c>
-      <c r="C23" s="1" t="s">
+      <c r="C23" s="21" t="s">
         <v>107</v>
       </c>
-      <c r="D23" s="1" t="s">
+      <c r="D23" s="21" t="s">
         <v>108</v>
       </c>
-      <c r="E23" s="1" t="s">
+      <c r="E23" s="21" t="s">
         <v>109</v>
       </c>
-      <c r="F23" s="4" t="s">
+      <c r="F23" s="23" t="s">
         <v>110</v>
       </c>
     </row>
     <row r="24" spans="1:6" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A24" s="3" t="s">
+      <c r="A24" s="20" t="s">
         <v>111</v>
       </c>
-      <c r="B24" s="1" t="s">
+      <c r="B24" s="21" t="s">
         <v>6</v>
       </c>
-      <c r="C24" s="2"/>
-      <c r="D24" s="1" t="s">
+      <c r="C24" s="22"/>
+      <c r="D24" s="21" t="s">
         <v>112</v>
       </c>
-      <c r="E24" s="1" t="s">
+      <c r="E24" s="21" t="s">
         <v>113</v>
       </c>
-      <c r="F24" s="4" t="s">
+      <c r="F24" s="23" t="s">
         <v>114</v>
       </c>
     </row>
     <row r="25" spans="1:6" ht="144" x14ac:dyDescent="0.3">
-      <c r="A25" s="3" t="s">
+      <c r="A25" s="20" t="s">
         <v>115</v>
       </c>
-      <c r="B25" s="2" t="s">
+      <c r="B25" s="22" t="s">
         <v>116</v>
       </c>
-      <c r="C25" s="1" t="s">
+      <c r="C25" s="21" t="s">
         <v>117</v>
       </c>
-      <c r="D25" s="1" t="s">
+      <c r="D25" s="21" t="s">
         <v>118</v>
       </c>
-      <c r="E25" s="1"/>
-      <c r="F25" s="4" t="s">
+      <c r="E25" s="21"/>
+      <c r="F25" s="23" t="s">
         <v>119</v>
       </c>
     </row>
     <row r="26" spans="1:6" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="A26" s="3" t="s">
+      <c r="A26" s="20" t="s">
         <v>120</v>
       </c>
-      <c r="B26" s="2" t="s">
+      <c r="B26" s="22" t="s">
         <v>121</v>
       </c>
-      <c r="C26" s="2"/>
-      <c r="D26" s="1" t="s">
+      <c r="C26" s="22"/>
+      <c r="D26" s="21" t="s">
         <v>122</v>
       </c>
-      <c r="E26" s="1" t="s">
+      <c r="E26" s="21" t="s">
         <v>123</v>
       </c>
-      <c r="F26" s="4" t="s">
+      <c r="F26" s="23" t="s">
         <v>124</v>
       </c>
     </row>
-    <row r="27" spans="1:6" ht="72.599999999999994" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A27" s="17" t="s">
+    <row r="27" spans="1:6" ht="72" x14ac:dyDescent="0.3">
+      <c r="A27" s="20" t="s">
         <v>125</v>
       </c>
-      <c r="B27" s="18" t="s">
+      <c r="B27" s="21" t="s">
         <v>6</v>
       </c>
-      <c r="C27" s="19"/>
-      <c r="D27" s="18" t="s">
+      <c r="C27" s="22"/>
+      <c r="D27" s="21" t="s">
         <v>126</v>
       </c>
-      <c r="E27" s="18" t="s">
+      <c r="E27" s="21" t="s">
         <v>127</v>
       </c>
-      <c r="F27" s="20" t="s">
+      <c r="F27" s="23" t="s">
         <v>128</v>
+      </c>
+    </row>
+    <row r="28" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A28" s="7" t="s">
+        <v>133</v>
+      </c>
+      <c r="B28" s="8" t="s">
+        <v>6</v>
+      </c>
+      <c r="C28" s="9"/>
+      <c r="D28" s="8" t="s">
+        <v>134</v>
+      </c>
+      <c r="E28" s="8" t="s">
+        <v>135</v>
+      </c>
+      <c r="F28" s="10" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="29" spans="1:6" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A29" s="7" t="s">
+        <v>137</v>
+      </c>
+      <c r="B29" s="9" t="s">
+        <v>55</v>
+      </c>
+      <c r="C29" s="8" t="s">
+        <v>107</v>
+      </c>
+      <c r="D29" s="8" t="s">
+        <v>138</v>
+      </c>
+      <c r="E29" s="8"/>
+      <c r="F29" s="10" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="30" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A30" s="7" t="s">
+        <v>140</v>
+      </c>
+      <c r="B30" s="8" t="s">
+        <v>6</v>
+      </c>
+      <c r="C30" s="9"/>
+      <c r="D30" s="8" t="s">
+        <v>141</v>
+      </c>
+      <c r="E30" s="8" t="s">
+        <v>142</v>
+      </c>
+      <c r="F30" s="10" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="31" spans="1:6" ht="72" x14ac:dyDescent="0.3">
+      <c r="A31" s="7" t="s">
+        <v>150</v>
+      </c>
+      <c r="B31" s="9" t="s">
+        <v>64</v>
+      </c>
+      <c r="C31" s="8" t="s">
+        <v>149</v>
+      </c>
+      <c r="D31" s="9" t="s">
+        <v>148</v>
+      </c>
+      <c r="E31" s="8"/>
+      <c r="F31" s="10" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="32" spans="1:6" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A32" s="7" t="s">
+        <v>151</v>
+      </c>
+      <c r="B32" s="8" t="s">
+        <v>6</v>
+      </c>
+      <c r="C32" s="9"/>
+      <c r="D32" s="8" t="s">
+        <v>147</v>
+      </c>
+      <c r="E32" s="11" t="s">
+        <v>146</v>
+      </c>
+      <c r="F32" s="10" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="33" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A33" s="12" t="s">
+        <v>152</v>
+      </c>
+      <c r="B33" s="13"/>
+      <c r="C33" s="13"/>
+      <c r="D33" s="13" t="s">
+        <v>153</v>
+      </c>
+      <c r="E33" s="14" t="s">
+        <v>154</v>
+      </c>
+      <c r="F33" s="15" t="s">
+        <v>155</v>
       </c>
     </row>
   </sheetData>

</xml_diff>